<commit_message>
data(ppc): cierra semana 08 (PPC 63%)
16 metas: 10 cumplidas / 6 no cumplidas. Enlaza el cierre en index.json,
agrega acta de cierre (PDF) y JSON de cierre; actualiza metas semana 08.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ppc/metas/semana-08.xlsx
+++ b/data/ppc/metas/semana-08.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e685dc9ab05c5d49/03. EZ PROJECT MANAGEMENT/06. CLAUDE CODE/06. ALTOZANO - TABLERO GENERAL/data/ppc/metas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="8_{E4D332A7-640B-4BBA-A73C-8CE23FBAEF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ADC24270-C7FD-425C-8393-6DEBE42708A9}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="8_{E4D332A7-640B-4BBA-A73C-8CE23FBAEF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1EE9ECE-B62D-44BC-B41F-D19A9A69D765}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -192,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -208,9 +208,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -677,7 +674,7 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="4" t="s">
         <v>23</v>
       </c>
       <c r="B15" s="3" t="s">
@@ -688,7 +685,7 @@
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="4" t="s">
         <v>26</v>
       </c>
       <c r="B16" s="3" t="s">

</xml_diff>